<commit_message>
polish(import): add date validation + input prompts (date YYYY-MM-DD, %, dropdown hints) — Excel's best for guided entry without macros
</commit_message>
<xml_diff>
--- a/templates/import_template.xlsx
+++ b/templates/import_template.xlsx
@@ -1178,7 +1178,7 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C4:C63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C4:C63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="幣別" prompt="請從下拉選單選擇" type="list">
       <formula1>"USD,TWD,HKD,EUR,JPY,CNY"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2514,14 +2514,42 @@
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
   </mergeCells>
-  <dataValidations count="3">
-    <dataValidation sqref="B4:B63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="10">
+    <dataValidation sqref="B4:B63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="類別" prompt="請從下拉選單選擇" type="list">
       <formula1>"SN,台股,期貨,美股,港股,國內外基金,ELN,PGN,儲蓄險,旅平險,車險,意外險"</formula1>
     </dataValidation>
-    <dataValidation sqref="M4:M63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I4:I63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="KO障壁 (%)" prompt="填數字即可（例 KO=100、票息=8 代表 8%）" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>100000</formula2>
+    </dataValidation>
+    <dataValidation sqref="J4:J63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="KI障壁 (%)" prompt="填數字即可（例 KO=100、票息=8 代表 8%）" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>100000</formula2>
+    </dataValidation>
+    <dataValidation sqref="K4:K63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="履約價 (%)" prompt="填數字即可（例 KO=100、票息=8 代表 8%）" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>100000</formula2>
+    </dataValidation>
+    <dataValidation sqref="L4:L63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="票息 (%年化)" prompt="填數字即可（例 KO=100、票息=8 代表 8%）" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>100000</formula2>
+    </dataValidation>
+    <dataValidation sqref="M4:M63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="配息頻率" prompt="請從下拉選單選擇" type="list">
       <formula1>"月配,季配,半年配,年配,到期一次"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q4:Q63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N4:N63" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="日期格式不正確" error="請用 YYYY-MM-DD（例 2026-06-18）" promptTitle="成交日" prompt="請輸入日期，格式 YYYY-MM-DD（例 2026-06-18）" type="date" operator="between">
+      <formula1>2000-01-01</formula1>
+      <formula2>2100-12-31</formula2>
+    </dataValidation>
+    <dataValidation sqref="O4:O63" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="日期格式不正確" error="請用 YYYY-MM-DD（例 2026-06-18）" promptTitle="比價日" prompt="請輸入日期，格式 YYYY-MM-DD（例 2026-06-18）" type="date" operator="between">
+      <formula1>2000-01-01</formula1>
+      <formula2>2100-12-31</formula2>
+    </dataValidation>
+    <dataValidation sqref="P4:P63" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="日期格式不正確" error="請用 YYYY-MM-DD（例 2026-06-18）" promptTitle="到期日" prompt="請輸入日期，格式 YYYY-MM-DD（例 2026-06-18）" type="date" operator="between">
+      <formula1>2000-01-01</formula1>
+      <formula2>2100-12-31</formula2>
+    </dataValidation>
+    <dataValidation sqref="Q4:Q63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="狀態" prompt="請從下拉選單選擇" type="list">
       <formula1>"進行中,已出場,暫停"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2960,7 +2988,7 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="D4:D63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D4:D63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="幣別" prompt="請從下拉選單選擇" type="list">
       <formula1>"USD,TWD,HKD,EUR,JPY,CNY"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(import): linked dropdowns (投資 picks investor/product from their sheets — no re-typing) + common-ticker list for 標的; recolor template dark green + gold (auspicious)
</commit_message>
<xml_diff>
--- a/templates/import_template.xlsx
+++ b/templates/import_template.xlsx
@@ -12,7 +12,10 @@
     <sheet name="商品" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="投資" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="InvestorList">'客戶'!$A$4:$A$63</definedName>
+    <definedName name="ProductList">'商品'!$A$4:$A$63</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -38,13 +41,13 @@
     </font>
     <font>
       <name val="Microsoft JhengHei"/>
-      <color rgb="001F1B1B"/>
+      <color rgb="001F2A24"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Microsoft JhengHei"/>
       <b val="1"/>
-      <color rgb="008E232E"/>
+      <color rgb="00153A2B"/>
       <sz val="12"/>
     </font>
     <font>
@@ -55,7 +58,7 @@
     </font>
     <font>
       <name val="Microsoft JhengHei"/>
-      <color rgb="008E232E"/>
+      <color rgb="00153A2B"/>
       <sz val="10"/>
     </font>
     <font>
@@ -67,7 +70,7 @@
     <font>
       <name val="Microsoft JhengHei"/>
       <i val="1"/>
-      <color rgb="008A7E7C"/>
+      <color rgb="006E827A"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -80,17 +83,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A62A36"/>
+        <fgColor rgb="001F4D3A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FBEEEF"/>
+        <fgColor rgb="00E9F2EC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="008E232E"/>
+        <fgColor rgb="00153A2B"/>
       </patternFill>
     </fill>
     <fill>
@@ -100,7 +103,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FAF7F7"/>
+        <fgColor rgb="00F4F9F6"/>
       </patternFill>
     </fill>
     <fill>
@@ -119,16 +122,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00EADDDB"/>
+        <color rgb="00D4E5DA"/>
       </left>
       <right style="thin">
-        <color rgb="00EADDDB"/>
+        <color rgb="00D4E5DA"/>
       </right>
       <top style="thin">
-        <color rgb="00EADDDB"/>
+        <color rgb="00D4E5DA"/>
       </top>
       <bottom style="thin">
-        <color rgb="00EADDDB"/>
+        <color rgb="00D4E5DA"/>
       </bottom>
     </border>
   </borders>
@@ -2514,7 +2517,7 @@
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
   </mergeCells>
-  <dataValidations count="10">
+  <dataValidations count="13">
     <dataValidation sqref="B4:B63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="類別" prompt="請從下拉選單選擇" type="list">
       <formula1>"SN,台股,期貨,美股,港股,國內外基金,ELN,PGN,儲蓄險,旅平險,車險,意外險"</formula1>
     </dataValidation>
@@ -2552,6 +2555,15 @@
     <dataValidation sqref="Q4:Q63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="狀態" prompt="請從下拉選單選擇" type="list">
       <formula1>"進行中,已出場,暫停"</formula1>
     </dataValidation>
+    <dataValidation sqref="C4:C63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" prompt="可選常用標的，或自行輸入其他代號" type="list">
+      <formula1>"NVDA,TSLA,TSM,ANET,AMD,INTC,AVGO,MSFT,ORCL,MU,GOOG,GOOGL,CRCL,LITE,COHR,QQQ,SPY,SMH,SOXX,IBB,AAPL,AMZN,META,NFLX"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" prompt="可選常用標的，或自行輸入其他代號" type="list">
+      <formula1>"NVDA,TSLA,TSM,ANET,AMD,INTC,AVGO,MSFT,ORCL,MU,GOOG,GOOGL,CRCL,LITE,COHR,QQQ,SPY,SMH,SOXX,IBB,AAPL,AMZN,META,NFLX"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G4:G63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" prompt="可選常用標的，或自行輸入其他代號" type="list">
+      <formula1>"NVDA,TSLA,TSM,ANET,AMD,INTC,AVGO,MSFT,ORCL,MU,GOOG,GOOGL,CRCL,LITE,COHR,QQQ,SPY,SMH,SOXX,IBB,AAPL,AMZN,META,NFLX"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2987,9 +2999,15 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="3">
     <dataValidation sqref="D4:D63" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="幣別" prompt="請從下拉選單選擇" type="list">
       <formula1>"USD,TWD,HKD,EUR,JPY,CNY"</formula1>
+    </dataValidation>
+    <dataValidation sqref="A4:A63" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="從「客戶」分頁選擇，不必重打" type="list">
+      <formula1>InvestorList</formula1>
+    </dataValidation>
+    <dataValidation sqref="B4:B63" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="從「商品」分頁選擇，不必重打" type="list">
+      <formula1>ProductList</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>